<commit_message>
content(printables): one label per field, and monolingual body text
- student-ai-use-process-sheet (English): every field description was printed
  twice — the English label and the gloss that survived from the Chinese
  edition. Each prints once now.
- student-ai-use-process-sheet (Chinese): the box descriptions, the rule and the
  box-4 note carried an English sentence each. The body is Chinese only; the
  fill-in field labels (姓名 Name: …) stay bilingual, which is the one bilingual
  element the house style allows.
- first-ai-lesson-kit, family-ai-homework-guide, maths-hint-cards-teacher-controlled
  (Chinese): the lines a person actually writes in now label their fields in both
  languages.
- one-term-ai-education-plan, p4-p6-curriculum-gap-map (Chinese): the fill-in
  column headers carry the English word beside the Chinese, matching the English
  editions.
</commit_message>
<xml_diff>
--- a/public/files/one-term-ai-education-plan.xlsx
+++ b/public/files/one-term-ai-education-plan.xlsx
@@ -479,6 +479,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -487,12 +488,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>負責人</t>
+          <t>負責人 Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>日期／週次</t>
+          <t>日期／週次 Dates / week</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -519,6 +520,7 @@
       <c r="C8" s="3" t="inlineStr"/>
       <c r="D8" s="3" t="inlineStr"/>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -526,6 +528,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
@@ -629,6 +632,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
@@ -637,12 +641,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>負責人</t>
+          <t>負責人 Owner</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>日期／週次</t>
+          <t>日期／週次 Dates / week</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -717,6 +721,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
@@ -724,6 +729,7 @@
         </is>
       </c>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>

</xml_diff>